<commit_message>
Updated excel file 26/09/2026
</commit_message>
<xml_diff>
--- a/12617630.xlsx
+++ b/12617630.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\India\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\India\Documents\ComputerApplication\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE6898F4-69C3-4BA0-B4DC-C91E12AD8ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6E87EE-6CE4-4E9A-932F-A33FBB465D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="99">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3048,25 +3048,47 @@
       <c r="A50" s="13">
         <v>46291</v>
       </c>
-      <c r="B50" s="14"/>
-      <c r="C50" s="14"/>
-      <c r="D50" s="14"/>
-      <c r="E50" s="14"/>
-      <c r="F50" s="14"/>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="15" t="str">
+      <c r="B50" s="14">
+        <v>480</v>
+      </c>
+      <c r="C50" s="14">
+        <v>30</v>
+      </c>
+      <c r="D50" s="14">
+        <v>150</v>
+      </c>
+      <c r="E50" s="14">
+        <v>30</v>
+      </c>
+      <c r="F50" s="14">
+        <v>0</v>
+      </c>
+      <c r="G50" s="14">
+        <v>0</v>
+      </c>
+      <c r="H50" s="14">
+        <v>300</v>
+      </c>
+      <c r="I50" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J50" s="15" t="str">
+        <v>990</v>
+      </c>
+      <c r="J50" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="17"/>
+        <v>450</v>
+      </c>
+      <c r="K50" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="L50" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="M50" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="N50" s="17" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A51" s="13"/>

</xml_diff>